<commit_message>
feat: real dashboard kpi endpoints with tenant context and created_at column
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-07</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -485,29 +485,29 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G2" t="n">
         <v>50.5</v>
       </c>
       <c r="H2" t="n">
-        <v>303</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -521,19 +521,19 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
         <v>200</v>
       </c>
       <c r="H3" t="n">
-        <v>1800</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-08</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -548,208 +548,208 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>150</v>
+        <v>50.5</v>
       </c>
       <c r="H4" t="n">
-        <v>1050</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H5" t="n">
-        <v>1800</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G6" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H6" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-02-14</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H7" t="n">
-        <v>400</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G8" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H8" t="n">
-        <v>404</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H9" t="n">
-        <v>303</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -764,38 +764,38 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H10" t="n">
-        <v>600</v>
+        <v>454.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -809,55 +809,55 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
         <v>200</v>
       </c>
       <c r="H11" t="n">
-        <v>800</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G12" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H12" t="n">
-        <v>101</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -881,55 +881,55 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
         <v>50.5</v>
       </c>
       <c r="H13" t="n">
-        <v>303</v>
+        <v>151.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H14" t="n">
-        <v>600</v>
+        <v>750</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -953,173 +953,173 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G15" t="n">
         <v>50.5</v>
       </c>
       <c r="H15" t="n">
-        <v>101</v>
+        <v>454.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G16" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H16" t="n">
-        <v>101</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G17" t="n">
-        <v>150</v>
+        <v>50.5</v>
       </c>
       <c r="H17" t="n">
-        <v>300</v>
+        <v>252.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G18" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H18" t="n">
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H19" t="n">
-        <v>151.5</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1133,29 +1133,29 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G20" t="n">
         <v>150</v>
       </c>
       <c r="H20" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1169,55 +1169,55 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
         <v>150</v>
       </c>
       <c r="H21" t="n">
-        <v>750</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G22" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H22" t="n">
-        <v>2000</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1232,28 +1232,28 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G23" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H23" t="n">
-        <v>1200</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1268,38 +1268,38 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G24" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H24" t="n">
-        <v>1400</v>
+        <v>151.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1313,19 +1313,19 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G25" t="n">
         <v>200</v>
       </c>
       <c r="H25" t="n">
-        <v>600</v>
+        <v>400</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1340,110 +1340,110 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H26" t="n">
-        <v>400</v>
+        <v>150</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G27" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H27" t="n">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-03-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H28" t="n">
-        <v>1200</v>
+        <v>300</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1457,29 +1457,29 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G29" t="n">
         <v>50.5</v>
       </c>
       <c r="H29" t="n">
-        <v>101</v>
+        <v>303</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1493,173 +1493,173 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G30" t="n">
         <v>150</v>
       </c>
       <c r="H30" t="n">
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H31" t="n">
-        <v>50.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G32" t="n">
-        <v>150</v>
+        <v>50.5</v>
       </c>
       <c r="H32" t="n">
-        <v>1050</v>
+        <v>303</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G33" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H33" t="n">
-        <v>303</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H34" t="n">
-        <v>505</v>
+        <v>150</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1673,65 +1673,65 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G35" t="n">
         <v>50.5</v>
       </c>
       <c r="H35" t="n">
-        <v>101</v>
+        <v>303</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-03-07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G36" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H36" t="n">
-        <v>454.5</v>
+        <v>400</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-01-17</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1745,19 +1745,19 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G37" t="n">
         <v>150</v>
       </c>
       <c r="H37" t="n">
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1772,64 +1772,64 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G38" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H38" t="n">
-        <v>454.5</v>
+        <v>400</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G39" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H39" t="n">
-        <v>400</v>
+        <v>750</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1844,28 +1844,28 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G40" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H40" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-22</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1880,28 +1880,28 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H41" t="n">
-        <v>101</v>
+        <v>450</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1925,19 +1925,19 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G42" t="n">
         <v>150</v>
       </c>
       <c r="H42" t="n">
-        <v>1200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1952,64 +1952,64 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G43" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H43" t="n">
-        <v>303</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G44" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H44" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2024,38 +2024,38 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G45" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H45" t="n">
-        <v>101</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2069,29 +2069,29 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G46" t="n">
         <v>50.5</v>
       </c>
       <c r="H46" t="n">
-        <v>101</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2105,29 +2105,29 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G47" t="n">
         <v>200</v>
       </c>
       <c r="H47" t="n">
-        <v>200</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2141,29 +2141,29 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G48" t="n">
         <v>150</v>
       </c>
       <c r="H48" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2189,7 +2189,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2204,28 +2204,28 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G50" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H50" t="n">
-        <v>353.5</v>
+        <v>200</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2240,100 +2240,100 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H51" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G52" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H52" t="n">
-        <v>1350</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G53" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H53" t="n">
-        <v>50.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2348,28 +2348,28 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G54" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H54" t="n">
-        <v>252.5</v>
+        <v>400</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2384,28 +2384,28 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G55" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H55" t="n">
-        <v>2000</v>
+        <v>151.5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2429,19 +2429,19 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G56" t="n">
         <v>50.5</v>
       </c>
       <c r="H56" t="n">
-        <v>505</v>
+        <v>101</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2465,55 +2465,55 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G57" t="n">
         <v>150</v>
       </c>
       <c r="H57" t="n">
-        <v>450</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G58" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H58" t="n">
-        <v>1350</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2528,100 +2528,100 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G59" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H59" t="n">
-        <v>505</v>
+        <v>600</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G60" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H60" t="n">
-        <v>454.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-01-11</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G61" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H61" t="n">
-        <v>800</v>
+        <v>252.5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-07</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2636,28 +2636,28 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G62" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H62" t="n">
-        <v>800</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2672,28 +2672,28 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F63" t="n">
         <v>9</v>
       </c>
       <c r="G63" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H63" t="n">
-        <v>1800</v>
+        <v>454.5</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2708,64 +2708,64 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G64" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H64" t="n">
-        <v>1050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H65" t="n">
-        <v>800</v>
+        <v>101</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2801,17 +2801,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-01-04</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2825,65 +2825,65 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G67" t="n">
         <v>50.5</v>
       </c>
       <c r="H67" t="n">
-        <v>404</v>
+        <v>505</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F68" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G68" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H68" t="n">
-        <v>600</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2897,19 +2897,19 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G69" t="n">
         <v>50.5</v>
       </c>
       <c r="H69" t="n">
-        <v>454.5</v>
+        <v>303</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2945,43 +2945,43 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F71" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G71" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H71" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2996,28 +2996,28 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G72" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H72" t="n">
-        <v>1600</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3032,28 +3032,28 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G73" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H73" t="n">
-        <v>505</v>
+        <v>900</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3068,28 +3068,28 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F74" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G74" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H74" t="n">
-        <v>1600</v>
+        <v>900</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3104,74 +3104,74 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G75" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H75" t="n">
-        <v>404</v>
+        <v>200</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G76" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H76" t="n">
-        <v>404</v>
+        <v>600</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3185,29 +3185,29 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G77" t="n">
         <v>50.5</v>
       </c>
       <c r="H77" t="n">
-        <v>505</v>
+        <v>151.5</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3221,19 +3221,19 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G78" t="n">
         <v>50.5</v>
       </c>
       <c r="H78" t="n">
-        <v>50.5</v>
+        <v>303</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3257,65 +3257,65 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G79" t="n">
         <v>150</v>
       </c>
       <c r="H79" t="n">
-        <v>450</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F80" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G80" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H80" t="n">
-        <v>505</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3329,29 +3329,29 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G81" t="n">
         <v>50.5</v>
       </c>
       <c r="H81" t="n">
-        <v>252.5</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3365,65 +3365,65 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G82" t="n">
         <v>50.5</v>
       </c>
       <c r="H82" t="n">
-        <v>202</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F83" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>50.5</v>
+        <v>200</v>
       </c>
       <c r="H83" t="n">
-        <v>252.5</v>
+        <v>200</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-01-10</t>
+          <t>2026-01-24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -3437,29 +3437,29 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G84" t="n">
         <v>200</v>
       </c>
       <c r="H84" t="n">
-        <v>1400</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3473,65 +3473,65 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G85" t="n">
         <v>150</v>
       </c>
       <c r="H85" t="n">
-        <v>300</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-03-14</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F86" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G86" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H86" t="n">
-        <v>600</v>
+        <v>353.5</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3545,101 +3545,101 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G87" t="n">
         <v>150</v>
       </c>
       <c r="H87" t="n">
-        <v>150</v>
+        <v>750</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P300</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto Z</t>
         </is>
       </c>
       <c r="F88" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G88" t="n">
-        <v>200</v>
+        <v>50.5</v>
       </c>
       <c r="H88" t="n">
-        <v>1800</v>
+        <v>353.5</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G89" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H89" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-02-17</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3665,7 +3665,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3689,29 +3689,29 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G91" t="n">
         <v>200</v>
       </c>
       <c r="H91" t="n">
-        <v>1600</v>
+        <v>800</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente C</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3725,19 +3725,19 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G92" t="n">
         <v>200</v>
       </c>
       <c r="H92" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-02-07</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3761,55 +3761,55 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G93" t="n">
         <v>150</v>
       </c>
       <c r="H93" t="n">
-        <v>450</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Cliente A</t>
+          <t>Cliente B</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F94" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G94" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H94" t="n">
-        <v>505</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3833,19 +3833,19 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G95" t="n">
         <v>50.5</v>
       </c>
       <c r="H95" t="n">
-        <v>252.5</v>
+        <v>454.5</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3869,91 +3869,91 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G96" t="n">
         <v>200</v>
       </c>
       <c r="H96" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Cliente C</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F97" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G97" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H97" t="n">
-        <v>800</v>
+        <v>900</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>P200</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Producto Y</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F98" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G98" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="H98" t="n">
-        <v>800</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-03-08</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3968,28 +3968,28 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G99" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H99" t="n">
-        <v>404</v>
+        <v>300</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4004,58 +4004,58 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>P100</t>
+          <t>P200</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Producto X</t>
+          <t>Producto Y</t>
         </is>
       </c>
       <c r="F100" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G100" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="H100" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Cliente B</t>
+          <t>Cliente A</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>P300</t>
+          <t>P100</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Producto Z</t>
+          <t>Producto X</t>
         </is>
       </c>
       <c r="F101" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G101" t="n">
-        <v>50.5</v>
+        <v>150</v>
       </c>
       <c r="H101" t="n">
-        <v>303</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>